<commit_message>
Update trace matrices to reflect v15-v16 fixes
- Book_Of_Quests: Solo quest abandonment → Fully Implemented, remove
  erroneous "All Loyal Knights dead" row (not in Book of Quests), fix
  traitor voluntary reveal description.
- rules_trace_matrix: Black Knight 2-pairs → Fully Implemented (v15),
  update instant-loss notes to reflect all-loyal-dead check in killKnight.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Book_Of_Quests_trace_matrix.xlsx
+++ b/Book_Of_Quests_trace_matrix.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -606,14 +606,14 @@
           <t>Solo Quests (Black Knight, Lancelot): only 1 Knight at a time. When a Knight leaves, white cards discarded, black cards remain. Quest not lost on abandonment.</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Partially Implemented</t>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Fully Implemented</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Solo restriction enforced via isSoloQuest()/isSoloQuestOccupied(). Guinevere forces solo white card removal. Voluntary abandonment with white card cleanup not explicitly triggered by player choice.</t>
+          <t>Solo restriction enforced via isSoloQuest()/isSoloQuestOccupied(). When a knight leaves a solo quest (move or Guinevere), all white cards are discarded; black cards remain.</t>
         </is>
       </c>
     </row>
@@ -1354,35 +1354,35 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>Sudden Defeat: All Loyal Knights dead = instant loss.</t>
-        </is>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>Not Yet Implemented</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>No code checks if all loyal knights are dead as a loss condition. Only individual knight death is handled.</t>
-        </is>
-      </c>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 13: KNIGHT SPECIAL POWERS</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="n"/>
+      <c r="C57" s="3" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 13: KNIGHT SPECIAL POWERS</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="n"/>
-      <c r="C58" s="3" t="n"/>
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>King Arthur: Exchange 1 White card face-down with any Knight regardless of location. Free action (not Heroic). Can be done before/after/between actions.</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Fully Implemented</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Multi-step UI: select card, select target, await return card. Free action, not consuming heroic.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>King Arthur: Exchange 1 White card face-down with any Knight regardless of location. Free action (not Heroic). Can be done before/after/between actions.</t>
+          <t>Sir Galahad: Play 1 Special White card for free (not Heroic Action). Must still take a different mandatory Heroic Action.</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
@@ -1392,14 +1392,14 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Multi-step UI: select card, select target, await return card. Free action, not consuming heroic.</t>
+          <t>galahadFreeSpecial heroic mode. galahadPowerUsed flag tracks once-per-turn.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Sir Galahad: Play 1 Special White card for free (not Heroic Action). Must still take a different mandatory Heroic Action.</t>
+          <t>Sir Gawain: Draw 3 instead of 2 at Round Table. Still subject to 12-card limit.</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
@@ -1409,14 +1409,14 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>galahadFreeSpecial heroic mode. galahadPowerUsed flag tracks once-per-turn.</t>
+          <t>Draw count = 3 when knight is gawain. Hand limit still enforced.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>Sir Gawain: Draw 3 instead of 2 at Round Table. Still subject to 12-card limit.</t>
+          <t>Sir Kay: Extra Fight card after Black cards revealed on Combat Quests. Also extra Fight card after die roll on Siege Engine fights.</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
@@ -1426,14 +1426,14 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Draw count = 3 when knight is gawain. Hand limit still enforced.</t>
+          <t>Kay bonus prompt appears at correct timing in both combat quest resolution and siege engine fights.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Sir Kay: Extra Fight card after Black cards revealed on Combat Quests. Also extra Fight card after die roll on Siege Engine fights.</t>
+          <t>Sir Palamedes: +1 extra LP per victorious Quest he is on. Max 6 LP.</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
@@ -1443,14 +1443,14 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Kay bonus prompt appears at correct timing in both combat quest resolution and siege engine fights.</t>
+          <t>Extra LP applied across all quest victory paths with Math.min(6,...) cap.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Sir Palamedes: +1 extra LP per victorious Quest he is on. Max 6 LP.</t>
+          <t>Sir Percival: Peek at top Black card before deciding whether to draw it or choose different Evil Action.</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
@@ -1460,14 +1460,14 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Extra LP applied across all quest victory paths with Math.min(6,...) cap.</t>
+          <t>Peek UI with percivalPeeked flag. Can then choose to draw or pick different evil action.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Sir Percival: Peek at top Black card before deciding whether to draw it or choose different Evil Action.</t>
+          <t>Sir Tristan: Departing Round Table is free (not Heroic Action). Gets another Heroic Action elsewhere.</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
@@ -1477,57 +1477,57 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Peek UI with percivalPeeked flag. Can then choose to draw or pick different evil action.</t>
+          <t>isTristanFree check allows free move from Round Table without consuming heroic action.</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t>Sir Tristan: Departing Round Table is free (not Heroic Action). Gets another Heroic Action elsewhere.</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>Fully Implemented</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>isTristanFree check allows free move from Round Table without consuming heroic action.</t>
-        </is>
-      </c>
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 14: THE TRAITOR</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="n"/>
+      <c r="C65" s="3" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 14: THE TRAITOR</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="n"/>
-      <c r="C66" s="3" t="n"/>
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>Hidden Traitor: plays normally, can lie about intent/resources, can falsely accuse a Loyal Knight.</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>Partially Implemented</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Hidden traitor plays normally and can falsely accuse. Voluntary reveal mentioned only in context of how traitor becomes revealed, not as explicit action rule.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Hidden Traitor: plays normally, can lie about intent/resources, can falsely accuse, can voluntarily reveal at any time.</t>
-        </is>
-      </c>
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>Partially Implemented</t>
+          <t>Revealed Traitor: miniature removed from board, Life die removed (cannot die), discard all White cards, Excalibur/Grail removed, Lancelot Armor stays.</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Fully Implemented</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Hidden traitor plays normally and can falsely accuse. Voluntary reveal button is not yet in the UI - reveal only occurs via accusation.</t>
+          <t>isRevealed flag set. Life die hidden. White cards cleared. Excalibur/Grail removed. Armor explicitly kept.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Revealed Traitor: miniature removed from board, Life die removed (cannot die), discard all White cards, Excalibur/Grail removed, Lancelot Armor stays.</t>
+          <t>Revealed Traitor Turn: 1) Taunt - steal 1 random White card from any Knight and discard it. 2) Choose: add 1 Siege Engine OR draw+play 1 Black card.</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
@@ -1537,40 +1537,40 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>isRevealed flag set. Life die hidden. White cards cleared. Excalibur/Grail removed. Armor explicitly kept.</t>
+          <t>Full revealed traitor turn flow with taunt (random card steal) and evil action choice.</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>Revealed Traitor Turn: 1) Taunt - steal 1 random White card from any Knight and discard it. 2) Choose: add 1 Siege Engine OR draw+play 1 Black card.</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="inlineStr">
-        <is>
-          <t>Fully Implemented</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>Full revealed traitor turn flow with taunt (random card steal) and evil action choice.</t>
-        </is>
-      </c>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 15: RELICS</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="n"/>
+      <c r="C69" s="3" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 15: RELICS</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="n"/>
-      <c r="C70" s="3" t="n"/>
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>Excalibur: +1 to Combat Quest and Siege Engine fight outcomes. Can cancel 1 Standard Black card just drawn (discard instead of placing). Cannot be gifted. Removed on Knight death.</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Fully Implemented</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>excaliburBonus in combat/siege. Cancel prompt on standard black draw. No gift mechanism. Removed on death.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Excalibur: +1 to Combat Quest and Siege Engine fight outcomes. Can cancel 1 Standard Black card just drawn (discard instead of placing). Cannot be gifted. Removed on Knight death.</t>
+          <t>Holy Grail: Dying Knight (0 LP) drinks, heals to 4 LP. Owner can use on self. Consumed after use. Cannot save revealed Traitor.</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
@@ -1580,14 +1580,14 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>excaliburBonus in combat/siege. Cancel prompt on standard black draw. No gift mechanism. Removed on death.</t>
+          <t>Grail save flow: offer prompt, heals to 4, removes relic. Self-use supported.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>Holy Grail: Dying Knight (0 LP) drinks, heals to 4 LP. Owner can use on self. Consumed after use. Cannot save revealed Traitor.</t>
+          <t>Lancelot Armor: Draw 2 Black cards instead of 1, play 1, put other back under pile. Stays with Traitor if revealed. Only relic that works for revealed Traitor.</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
@@ -1597,40 +1597,40 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Grail save flow: offer prompt, heals to 4, removes relic. Self-use supported.</t>
+          <t>Armor draw logic draws 2, player picks 1. Armor not removed on traitor reveal. Functions for revealed traitor.</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>Lancelot Armor: Draw 2 Black cards instead of 1, play 1, put other back under pile. Stays with Traitor if revealed. Only relic that works for revealed Traitor.</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>Fully Implemented</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>Armor draw logic draws 2, player picks 1. Armor not removed on traitor reveal. Functions for revealed traitor.</t>
-        </is>
-      </c>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 16: SPECIAL WHITE CARDS</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="n"/>
+      <c r="C73" s="3" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 16: SPECIAL WHITE CARDS</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="n"/>
-      <c r="C74" s="3" t="n"/>
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>Merlin (x7): Cancel - 3 Merlins collectively cancel 1 Special Black card when drawn (immediate, never retroactive). Heroic Play - remove 1 Siege Engine, or last Black card from a quest, or 1 warrior from Saxon/Pict War.</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Fully Implemented</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Multi-player Merlin contribution flow. All 3 heroic play options implemented.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>Merlin (x7): Cancel - 3 Merlins collectively cancel 1 Special Black card when drawn (immediate, never retroactive). Heroic Play - remove 1 Siege Engine, or last Black card from a quest, or 1 warrior from Saxon/Pict War.</t>
+          <t>Fate (x1): If Loyal, all Knights draw 1 White card. If Traitor, reveal self and all opponents discard 2 White cards.</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
@@ -1640,14 +1640,14 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Multi-player Merlin contribution flow. All 3 heroic play options implemented.</t>
+          <t>Loyalty-dependent branching. Loyal path draws for all. Traitor path forces reveal and discards.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>Fate (x1): If Loyal, all Knights draw 1 White card. If Traitor, reveal self and all opponents discard 2 White cards.</t>
+          <t>Piety (x1): Gain 3 LP (max 6) OR give 1 LP to every other Knight (max 6 each).</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
@@ -1657,14 +1657,14 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Loyalty-dependent branching. Loyal path draws for all. Traitor path forces reveal and discards.</t>
+          <t>Choice UI with both options. LP caps enforced.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>Piety (x1): Gain 3 LP (max 6) OR give 1 LP to every other Knight (max 6 each).</t>
+          <t>Heroism (x1): Place on Quest of choice. +1 White Sword if won, +1 Black Sword if lost.</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
@@ -1674,14 +1674,14 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Choice UI with both options. LP caps enforced.</t>
+          <t>Quest selection UI. Extra sword tracked and applied at quest resolution.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>Heroism (x1): Place on Quest of choice. +1 White Sword if won, +1 Black Sword if lost.</t>
+          <t>Reinforcements (x1): Draw 4 White cards for self OR let each other Knight draw 1.</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
@@ -1691,14 +1691,14 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Quest selection UI. Extra sword tracked and applied at quest resolution.</t>
+          <t>Both options with correct card distribution.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Reinforcements (x1): Draw 4 White cards for self OR let each other Knight draw 1.</t>
+          <t>Clairvoyance (x1): Draw top 5 Black cards, look at them, reorder as desired, place back on top.</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
@@ -1708,14 +1708,14 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Both options with correct card distribution.</t>
+          <t>Peek and reorder UI with drag/tap interface for 5 cards.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>Clairvoyance (x1): Draw top 5 Black cards, look at them, reorder as desired, place back on top.</t>
+          <t>Messenger (x1): Pass 1 to 3 White cards from hand to any Knight.</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
@@ -1725,14 +1725,14 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Peek and reorder UI with drag/tap interface for 5 cards.</t>
+          <t>Card selection (1-3) and target knight selection UI.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Messenger (x1): Pass 1 to 3 White cards from hand to any Knight.</t>
+          <t>Convocation (x1): All Knights return to Camelot. Draw White cards equal to number of Knights gathered and share.</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
@@ -1742,14 +1742,14 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Card selection (1-3) and target knight selection UI.</t>
+          <t>All knights moved to roundTable. Cards drawn = knight count, distributed.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>Convocation (x1): All Knights return to Camelot. Draw White cards equal to number of Knights gathered and share.</t>
+          <t>Lady of the Lake (x1): If Excalibur Quest in play, move Excalibur 1 step toward Knights. If quest completed, gain 2 LP instead.</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
@@ -1759,40 +1759,40 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>All knights moved to roundTable. Cards drawn = knight count, distributed.</t>
+          <t>Quest status check determines effect. Position adjusted or LP granted.</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="4" t="inlineStr">
-        <is>
-          <t>Lady of the Lake (x1): If Excalibur Quest in play, move Excalibur 1 step toward Knights. If quest completed, gain 2 LP instead.</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>Fully Implemented</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>Quest status check determines effect. Position adjusted or LP granted.</t>
-        </is>
-      </c>
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 17: STANDARD BLACK CARDS</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="n"/>
+      <c r="C83" s="3" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 17: STANDARD BLACK CARDS</t>
-        </is>
-      </c>
-      <c r="B84" s="3" t="n"/>
-      <c r="C84" s="3" t="n"/>
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>Black Knight Combat Cards (11): Values 1(x5), 3(x3), 5(x2), 7(x1). Placed face-down on quest. Revealed at resolution.</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Fully Implemented</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Card manifest matches. Cards placed on quest. Face-down until resolution.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Black Knight Combat Cards (11): Values 1(x5), 3(x3), 5(x2), 7(x1). Placed face-down on quest. Revealed at resolution.</t>
+          <t>Lancelot/Dragon Combat Cards (11): Dual values. Use Lancelot value when Lancelot active, Dragon value when Dragon active. Player may draw 1 free White card when placing face-down.</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
@@ -1802,14 +1802,14 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Card manifest matches. Cards placed on quest. Face-down until resolution.</t>
+          <t>Dual-value cards in manifest. Correct value used based on quest phase. Free white card draw on face-down placement.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>Lancelot/Dragon Combat Cards (11): Dual values. Use Lancelot value when Lancelot active, Dragon value when Dragon active. Player may draw 1 free White card when placing face-down.</t>
+          <t>Excalibur Cards (15): Move Excalibur 1 step toward Evil. Quest inactive = Siege Engine.</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
@@ -1819,14 +1819,14 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Dual-value cards in manifest. Correct value used based on quest phase. Free white card draw on face-down placement.</t>
+          <t>Position decremented. Inactive quest adds siege engine.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>Excalibur Cards (15): Move Excalibur 1 step toward Evil. Quest inactive = Siege Engine.</t>
+          <t>Despair Cards (15): Place on Holy Grail quest. Quest inactive = Siege Engine.</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
@@ -1836,14 +1836,14 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Position decremented. Inactive quest adds siege engine.</t>
+          <t>Card placed on quest board. Inactive quest adds siege engine.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>Despair Cards (15): Place on Holy Grail quest. Quest inactive = Siege Engine.</t>
+          <t>Mercenary (x4), Pict (x4), Saxon (x4): Add warriors. Mercenary is player choice. 4th warrior = immediate loss.</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
@@ -1853,40 +1853,40 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Card placed on quest board. Inactive quest adds siege engine.</t>
+          <t>Mercenary choice UI. Warrior count tracked. 4th warrior triggers war loss.</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="4" t="inlineStr">
-        <is>
-          <t>Mercenary (x4), Pict (x4), Saxon (x4): Add warriors. Mercenary is player choice. 4th warrior = immediate loss.</t>
-        </is>
-      </c>
-      <c r="B89" s="5" t="inlineStr">
-        <is>
-          <t>Fully Implemented</t>
-        </is>
-      </c>
-      <c r="C89" s="4" t="inlineStr">
-        <is>
-          <t>Mercenary choice UI. Warrior count tracked. 4th warrior triggers war loss.</t>
-        </is>
-      </c>
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 18: SPECIAL BLACK CARDS</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="n"/>
+      <c r="C89" s="3" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 18: SPECIAL BLACK CARDS</t>
-        </is>
-      </c>
-      <c r="B90" s="3" t="n"/>
-      <c r="C90" s="3" t="n"/>
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>All Special Black Cards (12 total): Applied immediately when drawn. Can be cancelled by 3 Merlin cards collectively (must be immediate, never retroactive).</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Fully Implemented</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>Merlin cancel flow triggers on all special black draws. 3-Merlin collective contribution system.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>All Special Black Cards (12 total): Applied immediately when drawn. Can be cancelled by 3 Merlin cards collectively (must be immediate, never retroactive).</t>
+          <t>Guinevere (x1): All Knights return to Camelot. Solo Quest white cards removed/discarded. Drawing player turn ends immediately.</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -1896,14 +1896,14 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Merlin cancel flow triggers on all special black draws. 3-Merlin collective contribution system.</t>
+          <t>All knights moved to roundTable. Solo quest whites cleared. Turn ended.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>Guinevere (x1): All Knights return to Camelot. Solo Quest white cards removed/discarded. Drawing player turn ends immediately.</t>
+          <t>Mist of Avalon (x1): Permanent. Each quest lost adds 1 extra Black Sword.</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
@@ -1913,14 +1913,14 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>All knights moved to roundTable. Solo quest whites cleared. Turn ended.</t>
+          <t>persistentEffects.mistOfAvalon flag. Extra black sword on quest loss.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Mist of Avalon (x1): Permanent. Each quest lost adds 1 extra Black Sword.</t>
+          <t>Mordred (x1): Add 1 warrior to Saxon or Pict War + attach Mordred. War needs extra Fight 5 to win. Removed on win/loss.</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -1930,14 +1930,14 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>persistentEffects.mistOfAvalon flag. Extra black sword on quest loss.</t>
+          <t>Choice panel for war selection. Mordred flag on war. Win threshold increased. Cleared on resolution.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>Mordred (x1): Add 1 warrior to Saxon or Pict War + attach Mordred. War needs extra Fight 5 to win. Removed on win/loss.</t>
+          <t>Vivien (x1): No Merlin cards may be played until a Quest is won. Can be cancelled by 3 Merlins when drawn.</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
@@ -1947,14 +1947,14 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Choice panel for war selection. Mordred flag on war. Win threshold increased. Cleared on resolution.</t>
+          <t>persistentEffects.vivien blocks Merlin play. Cleared on quest victory. Cancellable at draw time.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>Vivien (x1): No Merlin cards may be played until a Quest is won. Can be cancelled by 3 Merlins when drawn.</t>
+          <t>Morgan 1 (x1): Any Knight may volunteer to discard 3 cards. If nobody, each Knight discards 1.</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
@@ -1964,14 +1964,14 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>persistentEffects.vivien blocks Merlin play. Cleared on quest victory. Cancellable at draw time.</t>
+          <t>Volunteer prompt with timer/fallback. Both paths implemented.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>Morgan 1 (x1): Any Knight may volunteer to discard 3 cards. If nobody, each Knight discards 1.</t>
+          <t>Morgan 2 (x1): Drawing player draws and applies next 3 Black cards immediately.</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
@@ -1981,14 +1981,14 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>Volunteer prompt with timer/fallback. Both paths implemented.</t>
+          <t>morgan2Remaining counter. 3 successive black card draws.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>Morgan 2 (x1): Drawing player draws and applies next 3 Black cards immediately.</t>
+          <t>Morgan 3 (x1): Add 2 Siege Engines.</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
@@ -1998,14 +1998,14 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>morgan2Remaining counter. 3 successive black card draws.</t>
+          <t>Immediate +2 siege engines.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>Morgan 3 (x1): Add 2 Siege Engines.</t>
+          <t>Morgan 4 (x1): Each Knight loses 1 Life point.</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
@@ -2015,14 +2015,14 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Immediate +2 siege engines.</t>
+          <t>All alive knights lose 1 LP.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>Morgan 4 (x1): Each Knight loses 1 Life point.</t>
+          <t>Morgan 5 (x1): Any Knight may volunteer to lose 2 LP. If nobody, all Knights discard 1 White card each.</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
@@ -2032,14 +2032,14 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>All alive knights lose 1 LP.</t>
+          <t>Volunteer prompt. Both paths (2 LP loss or all discard 1) implemented.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>Morgan 5 (x1): Any Knight may volunteer to lose 2 LP. If nobody, all Knights discard 1 White card each.</t>
+          <t>Desolation (x2): Place on Holy Grail quest (special - only countered by 3 Merlins). If Holy Grail inactive, add Siege Engine.</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
@@ -2049,14 +2049,14 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Volunteer prompt. Both paths (2 LP loss or all discard 1) implemented.</t>
+          <t>Placed on grail board. Full-board replacement logic. Siege engine if quest inactive.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>Desolation (x2): Place on Holy Grail quest (special - only countered by 3 Merlins). If Holy Grail inactive, add Siege Engine.</t>
+          <t>Dark Forest (x1): No Grail cards may be played until a Quest is won. If Holy Grail inactive, add Siege Engine.</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
@@ -2066,40 +2066,40 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Placed on grail board. Full-board replacement logic. Siege engine if quest inactive.</t>
+          <t>persistentEffects.darkForest blocks grail play. Cleared on quest win. Siege engine if inactive.</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="4" t="inlineStr">
-        <is>
-          <t>Dark Forest (x1): No Grail cards may be played until a Quest is won. If Holy Grail inactive, add Siege Engine.</t>
-        </is>
-      </c>
-      <c r="B102" s="5" t="inlineStr">
-        <is>
-          <t>Fully Implemented</t>
-        </is>
-      </c>
-      <c r="C102" s="4" t="inlineStr">
-        <is>
-          <t>persistentEffects.darkForest blocks grail play. Cleared on quest win. Siege engine if inactive.</t>
-        </is>
-      </c>
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 19: CARDS MANIFEST</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="n"/>
+      <c r="C102" s="3" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 19: CARDS MANIFEST</t>
-        </is>
-      </c>
-      <c r="B103" s="3" t="n"/>
-      <c r="C103" s="3" t="n"/>
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>84 White cards: Fight 51 (1x14, 2x12, 3x10, 4x8, 5x7), Grail 18, Special 15 (Merlin x7, Fate x1, Piety x1, Heroism x1, Reinforcements x1, Clairvoyance x1, Messenger x1, Convocation x1, Lady of the Lake x1).</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Fully Implemented</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>CARD_MANIFEST in code matches all counts exactly.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>84 White cards: Fight 51 (1x14, 2x12, 3x10, 4x8, 5x7), Grail 18, Special 15 (Merlin x7, Fate x1, Piety x1, Heroism x1, Reinforcements x1, Clairvoyance x1, Messenger x1, Convocation x1, Lady of the Lake x1).</t>
+          <t>76 Black cards: BK 11, Lancelot/Dragon 11, Excalibur 15, Despair 15, Pict 4, Saxon 4, Mercenary 4, Special 12 (Morgan 1-5, Desolation x2, Dark Forest, Guinevere, Mist of Avalon, Mordred, Vivien).</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
@@ -2116,7 +2116,7 @@
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>76 Black cards: BK 11, Lancelot/Dragon 11, Excalibur 15, Despair 15, Pict 4, Saxon 4, Mercenary 4, Special 12 (Morgan 1-5, Desolation x2, Dark Forest, Guinevere, Mist of Avalon, Mordred, Vivien).</t>
+          <t>Hand limit: Max 12 White cards. Cannot draw at 12+. Hand can temporarily exceed 12 through Special card effects.</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
@@ -2126,66 +2126,66 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>CARD_MANIFEST in code matches all counts exactly.</t>
+          <t>getHandLimit() returns 12. Draw button disabled at limit. No active enforcement against special card overflow (permissive).</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="4" t="inlineStr">
-        <is>
-          <t>Hand limit: Max 12 White cards. Cannot draw at 12+. Hand can temporarily exceed 12 through Special card effects.</t>
-        </is>
-      </c>
-      <c r="B106" s="5" t="inlineStr">
-        <is>
-          <t>Fully Implemented</t>
-        </is>
-      </c>
-      <c r="C106" s="4" t="inlineStr">
-        <is>
-          <t>getHandLimit() returns 12. Draw button disabled at limit. No active enforcement against special card overflow (permissive).</t>
-        </is>
-      </c>
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 20: DECK RESHUFFLING</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="n"/>
+      <c r="C106" s="3" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 20: DECK RESHUFFLING</t>
-        </is>
-      </c>
-      <c r="B107" s="3" t="n"/>
-      <c r="C107" s="3" t="n"/>
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>When either draw pile (White or Black) runs out, reshuffle BOTH discard piles into fresh draw piles simultaneously.</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Fully Implemented</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>Both whiteDraw and blackDraw reshuffled from discards in same transaction when either runs out.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="4" t="inlineStr">
-        <is>
-          <t>When either draw pile (White or Black) runs out, reshuffle BOTH discard piles into fresh draw piles simultaneously.</t>
-        </is>
-      </c>
-      <c r="B108" s="5" t="inlineStr">
-        <is>
-          <t>Fully Implemented</t>
-        </is>
-      </c>
-      <c r="C108" s="4" t="inlineStr">
-        <is>
-          <t>Both whiteDraw and blackDraw reshuffled from discards in same transaction when either runs out.</t>
-        </is>
-      </c>
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>SECTION 21: PHYSICAL COMPONENTS &amp; LAYOUT</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="n"/>
+      <c r="C108" s="3" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>SECTION 21: PHYSICAL COMPONENTS &amp; LAYOUT</t>
-        </is>
-      </c>
-      <c r="B109" s="3" t="n"/>
-      <c r="C109" s="3" t="n"/>
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>Quest board illustrations, encounter indicator hexes, and physical token/miniature placement on game board.</t>
+        </is>
+      </c>
+      <c r="B109" s="8" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>Digital adaptation uses UI panels, icons, and state displays instead of physical board components.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>Quest board illustrations, encounter indicator hexes, and physical token/miniature placement on game board.</t>
+          <t>Coat of Arms reference card for each Knight showing Special Power summary.</t>
         </is>
       </c>
       <c r="B110" s="8" t="inlineStr">
@@ -2194,23 +2194,6 @@
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
-        <is>
-          <t>Digital adaptation uses UI panels, icons, and state displays instead of physical board components.</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="4" t="inlineStr">
-        <is>
-          <t>Coat of Arms reference card for each Knight showing Special Power summary.</t>
-        </is>
-      </c>
-      <c r="B111" s="8" t="inlineStr">
-        <is>
-          <t>Not Applicable</t>
-        </is>
-      </c>
-      <c r="C111" s="4" t="inlineStr">
         <is>
           <t>Digital version shows knight powers in UI. No physical reference card needed.</t>
         </is>

</xml_diff>